<commit_message>
425- download folder path change
</commit_message>
<xml_diff>
--- a/TestData/TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
+++ b/TestData/TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay.kumar\source\repos\SalesForce_Project\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VKumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A0521D-F298-491D-9119-E3305E89395E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE27DE68-DD68-499C-A89D-1E92BCDF7AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="548" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -301,9 +301,6 @@
     <t>ExportFileLocation</t>
   </si>
   <si>
-    <t>C:\Users\vijay.kumar\Downloads\</t>
-  </si>
-  <si>
     <t>ExportedFileName</t>
   </si>
   <si>
@@ -311,6 +308,9 @@
   </si>
   <si>
     <t>Kristian M. Whalen</t>
+  </si>
+  <si>
+    <t>C:\Users\VKumar0427\Downloads\</t>
   </si>
 </sst>
 </file>
@@ -661,13 +661,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -675,7 +675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -691,12 +691,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FBB8EB1-471A-4668-845A-6810E22F6BA4}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -704,7 +704,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -720,17 +720,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -743,17 +743,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -767,13 +767,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1398F625-8674-4D63-93D8-B47E3A580505}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -781,7 +781,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -789,10 +789,10 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" s="3"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J11" s="2"/>
     </row>
   </sheetData>
@@ -804,9 +804,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AD2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -898,7 +898,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -998,16 +998,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751812A8-ABA8-4232-9D81-14F299F55479}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1021,10 +1021,10 @@
         <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1035,10 +1035,10 @@
         <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1050,19 +1050,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>70</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G2" t="s">
         <v>22</v>
@@ -1122,13 +1122,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7552AB4B-37A5-4D47-8C03-7FFC70E2819F}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>

</xml_diff>